<commit_message>
refactor: merge partner_companies into entities table
Eliminate the partner_companies table (3 rows) by making partner
companies regular entities tagged 'partner' via entity_tags. Every
column was either redundant with entities (name, ruc, owner info)
or unused (bank_tracking_full). Reduces schema from 17 to 16 tables.

- Migration creates partner entities from live data, retargets FKs
- Rename partner_company_id → partner_id on 5 tables
- Update 7 views, fn_create_invoice_with_items, and all website code
- Regenerate TypeScript types and Excel import templates
- Update all documentation to reflect new schema

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/direct-transactions-template.xlsx
+++ b/website/public/templates/direct-transactions-template.xlsx
@@ -400,7 +400,7 @@
   <dimension ref="A1:I4"/>
   <cols>
     <col min="1" max="1" width="23.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
@@ -415,7 +415,7 @@
         <v>direction</v>
       </c>
       <c r="B1" t="str">
-        <v>partner_company_name</v>
+        <v>partner_name</v>
       </c>
       <c r="C1" t="str">
         <v>project_code</v>
@@ -444,7 +444,7 @@
         <v>Transaction direction</v>
       </c>
       <c r="B2" t="str">
-        <v>Partner company name</v>
+        <v>Partner name</v>
       </c>
       <c r="C2" t="str">
         <v>Project code</v>

</xml_diff>

<commit_message>
feat: auto-fill exchange rate from DB in direct transaction imports
exchange_rate is now optional in the direct-transactions Excel template.
When left blank, the import pulls the sell_rate from exchange_rates for
that row's date. Manual values still take precedence.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/direct-transactions-template.xlsx
+++ b/website/public/templates/direct-transactions-template.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="29.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
     <col min="9" max="9" width="21.83203125" customWidth="1"/>
   </cols>
@@ -517,7 +517,7 @@
         <v>USD, PEN</v>
       </c>
       <c r="G4" t="str">
-        <v>Required, 2.5–6.0</v>
+        <v>Optional — auto-filled from exchange_rates table if blank</v>
       </c>
       <c r="H4" t="str">
         <v>Required for outflow. Values: materials, labor, subcontractor, equipment_rental, permits_regulatory, other</v>

</xml_diff>

<commit_message>
feat: add document_ref to payments for payment receipt tracking
Add document_ref VARCHAR(100) to payments table, linking payment records
to physical receipts in SharePoint (PRY001-PY-001 convention). Update
v_payments_enriched view, Excel templates, import logic, and docs to
reflect new folder structure (merged 08-Facturas, new 09-ComprobantesPago).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/direct-transactions-template.xlsx
+++ b/website/public/templates/direct-transactions-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="23.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -407,7 +407,8 @@
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="7" width="40.83203125" customWidth="1"/>
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" customWidth="1"/>
+    <col min="9" max="9" width="27.83203125" customWidth="1"/>
+    <col min="10" max="10" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -436,6 +437,9 @@
         <v>category</v>
       </c>
       <c r="I1" t="str">
+        <v>document_ref</v>
+      </c>
+      <c r="J1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -465,6 +469,9 @@
         <v>Cost category (outflow only)</v>
       </c>
       <c r="I2" t="str">
+        <v>Payment receipt reference</v>
+      </c>
+      <c r="J2" t="str">
         <v>Notes / description</v>
       </c>
     </row>
@@ -494,6 +501,9 @@
         <v>materials</v>
       </c>
       <c r="I3" t="str">
+        <v>PRY001-PY-001</v>
+      </c>
+      <c r="J3" t="str">
         <v>Cash for nails</v>
       </c>
     </row>
@@ -520,15 +530,18 @@
         <v>Optional — auto-filled from exchange_rates table if blank</v>
       </c>
       <c r="H4" t="str">
-        <v>Required for outflow. Values: materials, labor, subcontractor, equipment_rental, permits_regulatory, other</v>
+        <v>Required for outflow. Values: materials, labor, subcontractor, equipment_rental, housing_food, other</v>
       </c>
       <c r="I4" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="J4" t="str">
         <v>Optional</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>